<commit_message>
V18 F6: Documento de Trabajo revisado (23 hallazgos del árbitro y los del verificador; K12); clases, periodos e indicadores de filas V18 corregidos en cifras_clave sin cambiar ningún valor (ERRATA)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GDwCFFTud391ebBMaJpdsw
</commit_message>
<xml_diff>
--- a/output/v18/documento/tablas_v18.xlsx
+++ b/output/v18/documento/tablas_v18.xlsx
@@ -236,7 +236,7 @@
     </comment>
     <comment ref="B11" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: output/v18/f5/magnitudes_estudios.csv; output/v18/f1/catalogo.csv; docs/v18/plan_replicacion_adenda.md (1.9). Origen: output/v18/f6/hechos.json:V18-B5-E8. Capa C4; clasificación V18: NO ESTIMABLE.</t>
+        <t>Fuente: output/v18/f5/magnitudes_estudios.csv; output/v18/f1/catalogo.csv; docs/v18/plan_replicacion_adenda.md (1.9). Origen: output/v18/f6/hechos.json:V18-B5-E8. Capa C4; clasificación V18: ASOCIACIÓN.</t>
       </text>
     </comment>
     <comment ref="I11" authorId="0" shapeId="0">
@@ -271,7 +271,7 @@
     </comment>
     <comment ref="A5" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: SERPAVI (MIVAU), alquiler mediano por sección, 2011-2024; Ajuntament de Barcelona, registro de viviendas de uso turístico (cortes trimestrales con coordenadas, data/manual/v11); INE, viviendas turísticas (INE-VUT) por sección; Censo 2021 (viviendas por sección); docs/v18/plan_replicacion.md + plan_replicacion_adenda.md (pre-registro interno plan-replicacion-v18). Origen: output/v18/f6/hechos.json:V18-E1-P-H3. Capa C4; clasificación V18: SUGESTIVO.</t>
+        <t>Fuente: SERPAVI (MIVAU), alquiler mediano por sección, 2011-2024; Ajuntament de Barcelona, registro de viviendas de uso turístico (cortes trimestrales con coordenadas, data/manual/v11); INE, viviendas turísticas (INE-VUT) por sección; Censo 2021 (viviendas por sección); docs/v18/plan_replicacion.md + plan_replicacion_adenda.md (pre-registro interno plan-replicacion-v18). Origen: output/v18/f6/hechos.json:V18-E1-P-H3. Capa C4; clasificación V18: sin clasificar (coprincipal informativa).</t>
       </text>
     </comment>
     <comment ref="A6" authorId="0" shapeId="0">
@@ -306,52 +306,52 @@
     </comment>
     <comment ref="A12" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-d-v1. Capa C4; clasificación V18: ASOCIACIÓN.</t>
+        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-d-v1. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A13" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-d-v2. Capa C4; clasificación V18: ASOCIACIÓN.</t>
+        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-d-v2. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A14" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-d-v3. Capa C4; clasificación V18: ASOCIACIÓN.</t>
+        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-d-v3. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A15" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-d-v4. Capa C4; clasificación V18: ASOCIACIÓN.</t>
+        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-d-v4. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A16" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-d-vF. Capa C4; clasificación V18: ASOCIACIÓN.</t>
+        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-d-vF. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A17" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-v1. Capa C4; clasificación V18: ASOCIACIÓN.</t>
+        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-v1. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A18" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-v2. Capa C4; clasificación V18: ASOCIACIÓN.</t>
+        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-v2. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A19" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-v3. Capa C4; clasificación V18: ASOCIACIÓN.</t>
+        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-v3. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A20" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-v4. Capa C4; clasificación V18: ASOCIACIÓN.</t>
+        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-v4. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A21" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-vF. Capa C4; clasificación V18: ASOCIACIÓN.</t>
+        <t>Fuente: base:serpavi_alquiler_m2_mediana municipal, vivienda colectiva (MIVAU/SERPAVI) 2019 y 2024; base:v12_titularidad_pct_mas10 y base:v12_titularidad_pct_pj municipales 2024 (Catastro; tramo contado dentro del municipio: cota inferior); base:adrh_renta_neta_persona por sección 2023 (promedio municipal); base:pob_censo_anual municipal 2024 (total); data/base/geo/municipios.parquet (centroides); output/v17/auditoria/oferta_titularidad_hechos.json (V17-AUD-OT-CAT-GT-PARQUE-2026). Origen: output/v18/f6/hechos.json:V18-E10-A1-vF. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A22" authorId="0" shapeId="0">
@@ -361,7 +361,7 @@
     </comment>
     <comment ref="A23" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: data/raw/mivau_v2_protegida.csv (calificaciones definitivas anuales de vivienda protegida, tabla 1.6, MIVAU); data/raw/mivau_v2_iniciadas_terminadas_prov.csv (viviendas libres iniciadas); data/raw/mivau_parque.csv (parque de viviendas); base:valor_tasado provincial y base:deflactor (E12-A2). Origen: output/v18/f6/hechos.json:V18-E12-A1-sin-atipicos. Capa C4; clasificación V18: NO ESTIMABLE.</t>
+        <t>Fuente: data/raw/mivau_v2_protegida.csv (calificaciones definitivas anuales de vivienda protegida, tabla 1.6, MIVAU); data/raw/mivau_v2_iniciadas_terminadas_prov.csv (viviendas libres iniciadas); data/raw/mivau_parque.csv (parque de viviendas); base:valor_tasado provincial y base:deflactor (E12-A2). Origen: output/v18/f6/hechos.json:V18-E12-A1-sin-atipicos. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A24" authorId="0" shapeId="0">
@@ -416,27 +416,27 @@
     </comment>
     <comment ref="A34" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); INE, Padrón municipal; IDESCAT (viviendas de uso turístico); INE, Censo 2021 (muestra del 10 %); docs/v18/revision_estimaciones/ronda1_e2_e8.md (ronda 1 del abogado del diablo). Origen: output/v18/f6/hechos.json:V18-E2-B6-A. Capa C4; clasificación V18: SUGESTIVO.</t>
+        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); INE, Padrón municipal; IDESCAT (viviendas de uso turístico); INE, Censo 2021 (muestra del 10 %); docs/v18/revision_estimaciones/ronda1_e2_e8.md (ronda 1 del abogado del diablo). Origen: output/v18/f6/hechos.json:V18-E2-B6-A. Capa C4; clasificación V18: robustez a posteriori.</t>
       </text>
     </comment>
     <comment ref="A35" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); INE, Padrón municipal; IDESCAT (viviendas de uso turístico); INE, Censo 2021 (muestra del 10 %); docs/v18/revision_estimaciones/ronda1_e2_e8.md (ronda 1 del abogado del diablo). Origen: output/v18/f6/hechos.json:V18-E2-B6-B. Capa C4; clasificación V18: SUGESTIVO.</t>
+        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); INE, Padrón municipal; IDESCAT (viviendas de uso turístico); INE, Censo 2021 (muestra del 10 %); docs/v18/revision_estimaciones/ronda1_e2_e8.md (ronda 1 del abogado del diablo). Origen: output/v18/f6/hechos.json:V18-E2-B6-B. Capa C4; clasificación V18: robustez a posteriori.</t>
       </text>
     </comment>
     <comment ref="A36" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); INE, Padrón municipal; IDESCAT (viviendas de uso turístico); INE, Censo 2021 (muestra del 10 %); docs/v18/revision_estimaciones/ronda1_e2_e8.md (ronda 1 del abogado del diablo). Origen: output/v18/f6/hechos.json:V18-E2-B6-C. Capa C4; clasificación V18: SUGESTIVO.</t>
+        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); INE, Padrón municipal; IDESCAT (viviendas de uso turístico); INE, Censo 2021 (muestra del 10 %); docs/v18/revision_estimaciones/ronda1_e2_e8.md (ronda 1 del abogado del diablo). Origen: output/v18/f6/hechos.json:V18-E2-B6-C. Capa C4; clasificación V18: robustez a posteriori.</t>
       </text>
     </comment>
     <comment ref="A37" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); INE, Padrón municipal; IDESCAT (viviendas de uso turístico); INE, Censo 2021 (muestra del 10 %); docs/v18/revision_estimaciones/ronda1_e2_e8.md (ronda 1 del abogado del diablo). Origen: output/v18/f6/hechos.json:V18-E2-B6-D. Capa C4; clasificación V18: SUGESTIVO.</t>
+        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); INE, Padrón municipal; IDESCAT (viviendas de uso turístico); INE, Censo 2021 (muestra del 10 %); docs/v18/revision_estimaciones/ronda1_e2_e8.md (ronda 1 del abogado del diablo). Origen: output/v18/f6/hechos.json:V18-E2-B6-D. Capa C4; clasificación V18: robustez a posteriori.</t>
       </text>
     </comment>
     <comment ref="A38" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); INE, Padrón municipal; IDESCAT (viviendas de uso turístico); INE, Censo 2021 (muestra del 10 %); docs/v18/revision_estimaciones/ronda1_e2_e8.md (ronda 1 del abogado del diablo). Origen: output/v18/f6/hechos.json:V18-E2-B6-R1CV1. Capa C4; clasificación V18: ASOCIACIÓN.</t>
+        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); INE, Padrón municipal; IDESCAT (viviendas de uso turístico); INE, Censo 2021 (muestra del 10 %); docs/v18/revision_estimaciones/ronda1_e2_e8.md (ronda 1 del abogado del diablo). Origen: output/v18/f6/hechos.json:V18-E2-B6-R1CV1. Capa C4; clasificación V18: robustez a posteriori.</t>
       </text>
     </comment>
     <comment ref="A39" authorId="0" shapeId="0">
@@ -446,7 +446,7 @@
     </comment>
     <comment ref="A40" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); docs/v18/plan_replicacion.md + plan_replicacion_adenda.md (pre-registro interno plan-replicacion-v18). Origen: output/v18/f6/hechos.json:V18-E2-R1-REV. Capa C4; clasificación V18: SUGESTIVO.</t>
+        <t>Fuente: Incasòl, fianzas (Socrata qww9-bvhh, descarga 2026-10-14); BOE-A-2020-11363 (Ley 11/2020 de Cataluña) y cataluna_contencion_rentas_v3.csv (v3); docs/v18/plan_replicacion.md + plan_replicacion_adenda.md (pre-registro interno plan-replicacion-v18). Origen: output/v18/f6/hechos.json:V18-E2-R1-REV. Capa C4; clasificación V18: diagnóstico o variante (sin clase propia).</t>
       </text>
     </comment>
     <comment ref="A41" authorId="0" shapeId="0">
@@ -1986,12 +1986,12 @@
     </comment>
     <comment ref="A222" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: output/v18/f5/contabilidad_ilustracion.csv; data/base/hechos.parquet; output/v18/f5/magnitudes.csv. Origen: output/v18/f6/hechos.json:V18-C5I-2020T1-2022T2-09-E2-extremos-N. Capa C4; clasificación V18: SUGESTIVO.</t>
+        <t>Fuente: output/v18/f5/contabilidad_ilustracion.csv; data/base/hechos.parquet; output/v18/f5/magnitudes.csv. Origen: output/v18/f6/hechos.json:V18-C5I-2020T1-2022T2-09-E2-extremos-N. Capa C4; clasificación V18: NO ESTIMABLE.</t>
       </text>
     </comment>
     <comment ref="A223" authorId="0" shapeId="0">
       <text>
-        <t>Fuente: output/v18/f5/contabilidad_ilustracion.csv; data/base/hechos.parquet; output/v18/f5/magnitudes.csv. Origen: output/v18/f6/hechos.json:V18-C5I-2020T1-2022T2-09-E2-vigencia-N. Capa C4; clasificación V18: SUGESTIVO.</t>
+        <t>Fuente: output/v18/f5/contabilidad_ilustracion.csv; data/base/hechos.parquet; output/v18/f5/magnitudes.csv. Origen: output/v18/f6/hechos.json:V18-C5I-2020T1-2022T2-09-E2-vigencia-N. Capa C4; clasificación V18: NO ESTIMABLE.</t>
       </text>
     </comment>
     <comment ref="A224" authorId="0" shapeId="0">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Magnitud preferida de topes al alquiler (E2): ATT en ln de la renta de los contratos regulados</t>
+          <t>Magnitud preferida de topes al alquiler (E2): diferencia en ln de la renta de los contratos regulados</t>
         </is>
       </c>
       <c r="D5" s="2" t="n"/>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>ATT en ln de la renta de los contratos regulados</t>
+          <t>diferencia en ln de la renta de los contratos regulados</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -3486,8 +3486,10 @@
       <c r="J10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="2" t="n">
-        <v/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>rango de 2 estudios (sanjuan_2023_bde_be2302art09, bce_eb_2022_6_battistini_gareis_roma)</t>
+        </is>
       </c>
       <c r="L10" s="6">
         <f>IF(AND(ISNUMBER(E10),ISNUMBER(F10)),F10-E10,"")</f>
@@ -3524,7 +3526,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>NO ESTIMABLE</t>
+          <t>ASOCIACIÓN</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -3535,8 +3537,10 @@
       <c r="J11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="2" t="n">
-        <v/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>rango de un solo estudio (dolls_etal_2020_vfs; valores de sus versiones o especificaciones)</t>
+        </is>
       </c>
       <c r="L11" s="6">
         <f>IF(AND(ISNUMBER(E11),ISNUMBER(F11)),F11-E11,"")</f>
@@ -3584,8 +3588,10 @@
       <c r="J12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="2" t="n">
-        <v/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>rango de un solo estudio (sa_2016_lse_cfm2016_39; valores de sus versiones o especificaciones)</t>
+        </is>
       </c>
       <c r="L12" s="6">
         <f>IF(AND(ISNUMBER(E12),ISNUMBER(F12)),F12-E12,"")</f>
@@ -3785,7 +3791,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>SUGESTIVO</t>
+          <t>sin clasificar (coprincipal informativa)</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -4190,7 +4196,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -4249,7 +4255,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -4308,7 +4314,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -4367,7 +4373,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -4426,7 +4432,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -4485,7 +4491,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -4544,7 +4550,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -4603,7 +4609,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -4662,7 +4668,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -4721,7 +4727,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -4835,7 +4841,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>NO ESTIMABLE</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -5444,7 +5450,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>SUGESTIVO</t>
+          <t>robustez a posteriori</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -5503,7 +5509,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>SUGESTIVO</t>
+          <t>robustez a posteriori</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -5562,7 +5568,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>SUGESTIVO</t>
+          <t>robustez a posteriori</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -5621,7 +5627,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>SUGESTIVO</t>
+          <t>robustez a posteriori</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -5680,7 +5686,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN</t>
+          <t>robustez a posteriori</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -5798,7 +5804,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>SUGESTIVO</t>
+          <t>diagnóstico o variante (sin clase propia)</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -10900,7 +10906,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 1995T1-2007T4, Nacional</t>
+          <t>Variación del alquiler real sin explicar, 2002T1-2007T4, Nacional</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -10919,7 +10925,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -11018,7 +11024,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 1995T1-2007T4, Andalucía</t>
+          <t>Variación del alquiler real sin explicar, 2002T1-2007T4, Andalucía (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -11037,7 +11043,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -11077,7 +11083,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 1995T1-2007T4, Andalucía</t>
+          <t>Variación del precio real sin explicar, 2002T1-2007T4, Andalucía (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -11096,7 +11102,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -11136,7 +11142,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 1995T1-2007T4, Castilla y León</t>
+          <t>Variación del alquiler real sin explicar, 2002T1-2007T4, Castilla y León (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -11155,7 +11161,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -11195,7 +11201,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 1995T1-2007T4, Castilla y León</t>
+          <t>Variación del precio real sin explicar, 2002T1-2007T4, Castilla y León (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -11214,7 +11220,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -11254,7 +11260,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 1995T1-2007T4, Castilla-La Mancha</t>
+          <t>Variación del alquiler real sin explicar, 2002T1-2007T4, Castilla-La Mancha (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -11273,7 +11279,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -11313,7 +11319,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 1995T1-2007T4, Castilla-La Mancha</t>
+          <t>Variación del precio real sin explicar, 2002T1-2007T4, Castilla-La Mancha (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -11332,7 +11338,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -11372,7 +11378,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 1995T1-2007T4, Cataluña</t>
+          <t>Variación del alquiler real sin explicar, 2002T1-2007T4, Cataluña (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -11391,7 +11397,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -11431,7 +11437,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 1995T1-2007T4, Cataluña</t>
+          <t>Variación del precio real sin explicar, 2002T1-2007T4, Cataluña (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -11450,7 +11456,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -11490,7 +11496,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 1995T1-2007T4, Comunitat Valenciana</t>
+          <t>Variación del alquiler real sin explicar, 2002T1-2007T4, Comunitat Valenciana (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -11509,7 +11515,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -11549,7 +11555,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 1995T1-2007T4, Comunitat Valenciana</t>
+          <t>Variación del precio real sin explicar, 1995T1-2007T4, Comunitat Valenciana (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -11608,7 +11614,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 1995T1-2007T4, Extremadura</t>
+          <t>Variación del alquiler real sin explicar, 2002T1-2007T4, Extremadura (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -11627,7 +11633,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -11667,7 +11673,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 1995T1-2007T4, Extremadura</t>
+          <t>Variación del precio real sin explicar, 2002T1-2007T4, Extremadura (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -11686,7 +11692,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -11726,7 +11732,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 1995T1-2007T4, Galicia</t>
+          <t>Variación del alquiler real sin explicar, 2002T1-2007T4, Galicia (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -11745,7 +11751,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -11785,7 +11791,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 1995T1-2007T4, Galicia</t>
+          <t>Variación del precio real sin explicar, 2002T1-2007T4, Galicia (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -11804,7 +11810,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -11844,7 +11850,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 1995T1-2007T4, País Vasco</t>
+          <t>Variación del alquiler real sin explicar, 2002T1-2007T4, País Vasco (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
@@ -11863,7 +11869,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -11903,7 +11909,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 1995T1-2007T4, País Vasco</t>
+          <t>Variación del precio real sin explicar, 2002T1-2007T4, País Vasco (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -11922,7 +11928,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>1995T1-2007T4</t>
+          <t>2002T1-2007T4</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -12080,7 +12086,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Andalucía</t>
+          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Andalucía (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -12139,7 +12145,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2008T1-2013T4, Andalucía</t>
+          <t>Variación del precio real sin explicar, 2008T1-2013T4, Andalucía (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
@@ -12198,7 +12204,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Castilla y León</t>
+          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Castilla y León (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
@@ -12257,7 +12263,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2008T1-2013T4, Castilla y León</t>
+          <t>Variación del precio real sin explicar, 2008T1-2013T4, Castilla y León (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -12316,7 +12322,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Castilla-La Mancha</t>
+          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Castilla-La Mancha (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -12375,7 +12381,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2008T1-2013T4, Castilla-La Mancha</t>
+          <t>Variación del precio real sin explicar, 2008T1-2013T4, Castilla-La Mancha (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
@@ -12434,7 +12440,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Cataluña</t>
+          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Cataluña (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
@@ -12493,7 +12499,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2008T1-2013T4, Cataluña</t>
+          <t>Variación del precio real sin explicar, 2008T1-2013T4, Cataluña (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
@@ -12552,7 +12558,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Comunitat Valenciana</t>
+          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Comunitat Valenciana (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -12611,7 +12617,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2008T1-2013T4, Comunitat Valenciana</t>
+          <t>Variación del precio real sin explicar, 2008T1-2013T4, Comunitat Valenciana (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
@@ -12670,7 +12676,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Extremadura</t>
+          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Extremadura (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -12729,7 +12735,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2008T1-2013T4, Extremadura</t>
+          <t>Variación del precio real sin explicar, 2008T1-2013T4, Extremadura (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -12788,7 +12794,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Galicia</t>
+          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, Galicia (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
@@ -12847,7 +12853,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2008T1-2013T4, Galicia</t>
+          <t>Variación del precio real sin explicar, 2008T1-2013T4, Galicia (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -12906,7 +12912,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, País Vasco</t>
+          <t>Variación del alquiler real sin explicar, 2008T1-2013T4, País Vasco (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -12965,7 +12971,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2008T1-2013T4, País Vasco</t>
+          <t>Variación del precio real sin explicar, 2008T1-2013T4, País Vasco (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -13142,7 +13148,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Andalucía</t>
+          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Andalucía (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
@@ -13201,7 +13207,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2014T1-2019T4, Andalucía</t>
+          <t>Variación del precio real sin explicar, 2014T1-2019T4, Andalucía (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -13260,7 +13266,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Castilla y León</t>
+          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Castilla y León (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
@@ -13319,7 +13325,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2014T1-2019T4, Castilla y León</t>
+          <t>Variación del precio real sin explicar, 2014T1-2019T4, Castilla y León (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
@@ -13378,7 +13384,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Castilla-La Mancha</t>
+          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Castilla-La Mancha (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -13437,7 +13443,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2014T1-2019T4, Castilla-La Mancha</t>
+          <t>Variación del precio real sin explicar, 2014T1-2019T4, Castilla-La Mancha (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
@@ -13496,7 +13502,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Cataluña</t>
+          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Cataluña (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
@@ -13555,7 +13561,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2014T1-2019T4, Cataluña</t>
+          <t>Variación del precio real sin explicar, 2014T1-2019T4, Cataluña (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -13614,7 +13620,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Comunitat Valenciana</t>
+          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Comunitat Valenciana (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
@@ -13673,7 +13679,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2014T1-2019T4, Comunitat Valenciana</t>
+          <t>Variación del precio real sin explicar, 2014T1-2019T4, Comunitat Valenciana (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -13732,7 +13738,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Extremadura</t>
+          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Extremadura (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
@@ -13791,7 +13797,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2014T1-2019T4, Extremadura</t>
+          <t>Variación del precio real sin explicar, 2014T1-2019T4, Extremadura (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
@@ -13850,7 +13856,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Galicia</t>
+          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, Galicia (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
@@ -13909,7 +13915,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2014T1-2019T4, Galicia</t>
+          <t>Variación del precio real sin explicar, 2014T1-2019T4, Galicia (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
@@ -13968,7 +13974,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, País Vasco</t>
+          <t>Variación del alquiler real sin explicar, 2014T1-2019T4, País Vasco (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
@@ -14027,7 +14033,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2014T1-2019T4, País Vasco</t>
+          <t>Variación del precio real sin explicar, 2014T1-2019T4, País Vasco (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
@@ -14204,7 +14210,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Andalucía</t>
+          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Andalucía (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
@@ -14263,7 +14269,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2020T1-2022T2, Andalucía</t>
+          <t>Variación del precio real sin explicar, 2020T1-2022T2, Andalucía (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -14322,7 +14328,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Castilla y León</t>
+          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Castilla y León (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
@@ -14381,7 +14387,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2020T1-2022T2, Castilla y León</t>
+          <t>Variación del precio real sin explicar, 2020T1-2022T2, Castilla y León (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
@@ -14440,7 +14446,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Castilla-La Mancha</t>
+          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Castilla-La Mancha (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
@@ -14499,7 +14505,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2020T1-2022T2, Castilla-La Mancha</t>
+          <t>Variación del precio real sin explicar, 2020T1-2022T2, Castilla-La Mancha (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
@@ -14558,7 +14564,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Cataluña</t>
+          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Cataluña (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -14617,7 +14623,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2020T1-2022T2, Cataluña</t>
+          <t>Variación del precio real sin explicar, 2020T1-2022T2, Cataluña (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
@@ -14676,7 +14682,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Comunitat Valenciana</t>
+          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Comunitat Valenciana (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
@@ -14735,7 +14741,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2020T1-2022T2, Comunitat Valenciana</t>
+          <t>Variación del precio real sin explicar, 2020T1-2022T2, Comunitat Valenciana (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -14794,7 +14800,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Extremadura</t>
+          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Extremadura (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
@@ -14853,7 +14859,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2020T1-2022T2, Extremadura</t>
+          <t>Variación del precio real sin explicar, 2020T1-2022T2, Extremadura (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
@@ -14912,7 +14918,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Galicia</t>
+          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, Galicia (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
@@ -14971,7 +14977,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2020T1-2022T2, Galicia</t>
+          <t>Variación del precio real sin explicar, 2020T1-2022T2, Galicia (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
@@ -15030,7 +15036,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, País Vasco</t>
+          <t>Variación del alquiler real sin explicar, 2020T1-2022T2, País Vasco (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
@@ -15089,7 +15095,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2020T1-2022T2, País Vasco</t>
+          <t>Variación del precio real sin explicar, 2020T1-2022T2, País Vasco (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
@@ -15266,7 +15272,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Andalucía</t>
+          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Andalucía (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
@@ -15325,7 +15331,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2022T3-2026T2, Andalucía</t>
+          <t>Variación del precio real sin explicar, 2022T3-2026T2, Andalucía (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
@@ -15384,7 +15390,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Castilla y León</t>
+          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Castilla y León (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -15443,7 +15449,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2022T3-2026T2, Castilla y León</t>
+          <t>Variación del precio real sin explicar, 2022T3-2026T2, Castilla y León (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
@@ -15502,7 +15508,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Castilla-La Mancha</t>
+          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Castilla-La Mancha (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
@@ -15561,7 +15567,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2022T3-2026T2, Castilla-La Mancha</t>
+          <t>Variación del precio real sin explicar, 2022T3-2026T2, Castilla-La Mancha (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
@@ -15620,7 +15626,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Cataluña</t>
+          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Cataluña (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
@@ -15679,7 +15685,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2022T3-2026T2, Cataluña</t>
+          <t>Variación del precio real sin explicar, 2022T3-2026T2, Cataluña (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
@@ -15738,7 +15744,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Comunitat Valenciana</t>
+          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Comunitat Valenciana (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
@@ -15797,7 +15803,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2022T3-2026T2, Comunitat Valenciana</t>
+          <t>Variación del precio real sin explicar, 2022T3-2026T2, Comunitat Valenciana (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
@@ -15856,7 +15862,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Extremadura</t>
+          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Extremadura (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
@@ -15915,7 +15921,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2022T3-2026T2, Extremadura</t>
+          <t>Variación del precio real sin explicar, 2022T3-2026T2, Extremadura (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
@@ -15974,7 +15980,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Galicia</t>
+          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, Galicia (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
@@ -16033,7 +16039,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2022T3-2026T2, Galicia</t>
+          <t>Variación del precio real sin explicar, 2022T3-2026T2, Galicia (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
@@ -16092,7 +16098,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, País Vasco</t>
+          <t>Variación del alquiler real sin explicar, 2022T3-2026T2, País Vasco (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
@@ -16151,7 +16157,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Variación del precio real sin explicar, 2022T3-2026T2, País Vasco</t>
+          <t>Variación del precio real sin explicar, 2022T3-2026T2, País Vasco (relativa a la media de las provincias no selladas, sin el componente común)</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
@@ -23796,7 +23802,7 @@
       </c>
       <c r="J222" s="2" t="inlineStr">
         <is>
-          <t>SUGESTIVO</t>
+          <t>NO ESTIMABLE</t>
         </is>
       </c>
       <c r="K222" s="2" t="inlineStr">
@@ -23855,7 +23861,7 @@
       </c>
       <c r="J223" s="2" t="inlineStr">
         <is>
-          <t>SUGESTIVO</t>
+          <t>NO ESTIMABLE</t>
         </is>
       </c>
       <c r="K223" s="2" t="inlineStr">

</xml_diff>